<commit_message>
bug: edición de métricas
</commit_message>
<xml_diff>
--- a/data/database/dimension_values.xlsx
+++ b/data/database/dimension_values.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,48 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pangui</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-03 23:33:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pullinque</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-03 23:33:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Introduce metric management feature with data models, backend API, and a frontend UI for defining and editing metrics, including data types and dimensions.
</commit_message>
<xml_diff>
--- a/data/database/dimension_values.xlsx
+++ b/data/database/dimension_values.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,6 +494,69 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>2026-02-03 23:33:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-03 23:56:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-03 23:56:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-03 23:56:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
inestable: Cambios en datos, de specs, nuevos pasos pipeline para solicitar enrich con datos de usuario
</commit_message>
<xml_diff>
--- a/data/database/dimension_values.xlsx
+++ b/data/database/dimension_values.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,14 +457,14 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="n">
         <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pangui</t>
+          <t>Pullinque</t>
         </is>
       </c>
       <c r="D2" t="b">
@@ -472,20 +472,20 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-02-03 23:33:39</t>
+          <t>2026-02-03 23:33:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3" t="n">
         <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pullinque</t>
+          <t>Panguipulli</t>
         </is>
       </c>
       <c r="D3" t="b">
@@ -493,13 +493,13 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-02-03 23:33:49</t>
+          <t>2026-02-12 12:05:44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="n">
         <v>5</v>
@@ -514,20 +514,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-02-03 23:56:14</t>
+          <t>2026-02-13 09:59:01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" t="n">
         <v>5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -535,20 +535,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-02-03 23:56:18</t>
+          <t>2026-02-13 09:59:03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -556,7 +556,28 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-02-03 23:56:21</t>
+          <t>2026-02-13 09:59:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2D</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-13 09:59:05</t>
         </is>
       </c>
     </row>

</xml_diff>